<commit_message>
update example, correct sheet viewports/selections
</commit_message>
<xml_diff>
--- a/odcs-template-v3.2.xlsx
+++ b/odcs-template-v3.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBACBCCE-EAC4-F945-B861-C87BF230602B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3951829-6F38-7B4C-88E7-5B20E0EEFA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="-33240" windowWidth="60160" windowHeight="33240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-33240" windowWidth="60160" windowHeight="33240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="8" r:id="rId1"/>
@@ -14370,10 +14370,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="5" t="str">
-        <f>IF(owner &lt;&gt; "", owner, "")</f>
-        <v/>
-      </c>
+      <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
         <v>48</v>
       </c>
@@ -14381,18 +14378,9 @@
         <f>IF(owner &lt;&gt; "", owner, "")</f>
         <v/>
       </c>
-      <c r="E5" s="5" t="str">
-        <f>IF(owner &lt;&gt; "", owner, "")</f>
-        <v/>
-      </c>
-      <c r="F5" s="5" t="str">
-        <f>IF(owner &lt;&gt; "", owner, "")</f>
-        <v/>
-      </c>
-      <c r="G5" s="5" t="str">
-        <f>IF(owner &lt;&gt; "", owner, "")</f>
-        <v/>
-      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>

</xml_diff>

<commit_message>
add logical type to schemas
</commit_message>
<xml_diff>
--- a/odcs-template-v3.2.xlsx
+++ b/odcs-template-v3.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3875D753-AACC-B04A-B375-AAA28B30B143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20183E6F-6333-DF4B-A803-E6DEE385A976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-33240" windowWidth="60160" windowHeight="33240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="8" r:id="rId1"/>
@@ -61,17 +61,18 @@
     <definedName name="quality">Quality!$A$4:$BF$300</definedName>
     <definedName name="relationships">Relationships!$A$4:$AZ$300</definedName>
     <definedName name="roles" localSheetId="7">Roles!$A$4:$AZ$1000</definedName>
-    <definedName name="schema.businessName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$8</definedName>
-    <definedName name="schema.context.instructions" localSheetId="2">'Schema &lt;table_name&gt;'!$B$13</definedName>
-    <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema &lt;table_name&gt;'!$B$10</definedName>
-    <definedName name="schema.deprecated" localSheetId="2">'Schema &lt;table_name&gt;'!$B$14</definedName>
-    <definedName name="schema.description" localSheetId="2">'Schema &lt;table_name&gt;'!$B$7</definedName>
-    <definedName name="schema.id" localSheetId="2">'Schema &lt;table_name&gt;'!$B$12</definedName>
+    <definedName name="schema.businessName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$9</definedName>
+    <definedName name="schema.context.instructions" localSheetId="2">'Schema &lt;table_name&gt;'!$B$14</definedName>
+    <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema &lt;table_name&gt;'!$B$11</definedName>
+    <definedName name="schema.deprecated" localSheetId="2">'Schema &lt;table_name&gt;'!$B$15</definedName>
+    <definedName name="schema.description" localSheetId="2">'Schema &lt;table_name&gt;'!$B$8</definedName>
+    <definedName name="schema.id" localSheetId="2">'Schema &lt;table_name&gt;'!$B$13</definedName>
+    <definedName name="schema.logicalType" localSheetId="2">'Schema &lt;table_name&gt;'!$B$7</definedName>
     <definedName name="schema.name" localSheetId="2">'Schema &lt;table_name&gt;'!$B$5</definedName>
-    <definedName name="schema.physicalName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$9</definedName>
+    <definedName name="schema.physicalName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$10</definedName>
     <definedName name="schema.physicalType" localSheetId="2">'Schema &lt;table_name&gt;'!$B$6</definedName>
-    <definedName name="schema.properties" localSheetId="2">'Schema &lt;table_name&gt;'!$A$16:$AW$984</definedName>
-    <definedName name="schema.tags" localSheetId="2">'Schema &lt;table_name&gt;'!$B$11</definedName>
+    <definedName name="schema.properties" localSheetId="2">'Schema &lt;table_name&gt;'!$A$17:$AW$985</definedName>
+    <definedName name="schema.tags" localSheetId="2">'Schema &lt;table_name&gt;'!$B$12</definedName>
     <definedName name="servers.account">Servers!$C$11</definedName>
     <definedName name="servers.catalog">Servers!$C$12</definedName>
     <definedName name="servers.catalogUrl">Servers!$C$13</definedName>
@@ -133,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="260">
   <si>
     <t>Property</t>
   </si>
@@ -1158,7 +1159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1246,12 +1247,6 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1262,6 +1257,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -15494,10 +15504,10 @@
       <c r="B12" s="7"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="35" t="s">
+      <c r="A13" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="36"/>
+      <c r="B13" s="43"/>
       <c r="C13" s="5"/>
       <c r="E13" s="6"/>
     </row>
@@ -15602,7 +15612,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AZ52"/>
+  <dimension ref="A1:AZ53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" style="2" customWidth="1"/>
@@ -15648,334 +15658,289 @@
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
+        <v>6</v>
+      </c>
+      <c r="B7" s="39"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="41"/>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="40"/>
+        <v>3</v>
+      </c>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" s="38"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40"/>
+        <v>9</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="38"/>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="40"/>
+        <v>51</v>
+      </c>
+      <c r="B10" s="36"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="38"/>
     </row>
     <row r="11" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="37"/>
+        <v>52</v>
+      </c>
+      <c r="B11" s="36"/>
       <c r="C11" s="37"/>
       <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
+      <c r="E11" s="38"/>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
+        <v>12</v>
+      </c>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
+        <v>22</v>
+      </c>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
     </row>
     <row r="14" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+    </row>
+    <row r="15" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-    </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="E15" s="2"/>
-      <c r="Y15" s="19" t="s">
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+    </row>
+    <row r="16" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="E16" s="2"/>
+      <c r="Y16" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="Z15" s="20"/>
-      <c r="AA15" s="20"/>
-      <c r="AB15" s="20"/>
-      <c r="AC15" s="20"/>
-      <c r="AD15" s="20"/>
-      <c r="AE15" s="20"/>
-      <c r="AF15" s="20"/>
-      <c r="AG15" s="20"/>
-      <c r="AH15" s="20"/>
-      <c r="AI15" s="20"/>
-      <c r="AJ15" s="20"/>
-      <c r="AK15" s="20"/>
-      <c r="AL15" s="20"/>
-      <c r="AM15" s="20"/>
-      <c r="AN15" s="20"/>
-      <c r="AO15" s="20"/>
-      <c r="AP15" s="20"/>
-      <c r="AQ15" s="20"/>
-      <c r="AR15" s="20"/>
-      <c r="AS15" s="20"/>
-      <c r="AT15" s="20"/>
-      <c r="AU15" s="21"/>
-      <c r="AX15" s="19" t="s">
+      <c r="Z16" s="20"/>
+      <c r="AA16" s="20"/>
+      <c r="AB16" s="20"/>
+      <c r="AC16" s="20"/>
+      <c r="AD16" s="20"/>
+      <c r="AE16" s="20"/>
+      <c r="AF16" s="20"/>
+      <c r="AG16" s="20"/>
+      <c r="AH16" s="20"/>
+      <c r="AI16" s="20"/>
+      <c r="AJ16" s="20"/>
+      <c r="AK16" s="20"/>
+      <c r="AL16" s="20"/>
+      <c r="AM16" s="20"/>
+      <c r="AN16" s="20"/>
+      <c r="AO16" s="20"/>
+      <c r="AP16" s="20"/>
+      <c r="AQ16" s="20"/>
+      <c r="AR16" s="20"/>
+      <c r="AS16" s="20"/>
+      <c r="AT16" s="20"/>
+      <c r="AU16" s="21"/>
+      <c r="AX16" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="AY15" s="20"/>
-      <c r="AZ15" s="20"/>
-    </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A16" s="9" t="s">
+      <c r="AY16" s="20"/>
+      <c r="AZ16" s="20"/>
+    </row>
+    <row r="17" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B17" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C17" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D17" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E17" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F17" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G17" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="10" t="s">
+      <c r="I17" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="J17" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="K16" s="10" t="s">
+      <c r="K17" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="L16" s="10" t="s">
+      <c r="L17" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="M16" s="10" t="s">
+      <c r="M17" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="N16" s="10" t="s">
+      <c r="N17" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="O16" s="10" t="s">
+      <c r="O17" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="P16" s="10" t="s">
+      <c r="P17" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="Q16" s="10" t="s">
+      <c r="Q17" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="R16" s="10" t="s">
+      <c r="R17" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="S16" s="10" t="s">
+      <c r="S17" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="T16" s="10" t="s">
+      <c r="T17" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="U16" s="10" t="s">
+      <c r="U17" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="V16" s="10" t="s">
+      <c r="V17" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="W16" s="10" t="s">
+      <c r="W17" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="X16" s="10" t="s">
+      <c r="X17" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="Y16" s="10" t="s">
+      <c r="Y17" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="Z16" s="10" t="s">
+      <c r="Z17" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="AA16" s="10" t="s">
+      <c r="AA17" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="AB16" s="10" t="s">
+      <c r="AB17" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="AC16" s="10" t="s">
+      <c r="AC17" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="AD16" s="10" t="s">
+      <c r="AD17" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="AE16" s="10" t="s">
+      <c r="AE17" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="AF16" s="10" t="s">
+      <c r="AF17" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="AG16" s="10" t="s">
+      <c r="AG17" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="AH16" s="10" t="s">
+      <c r="AH17" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="AI16" s="10" t="s">
+      <c r="AI17" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="AJ16" s="10" t="s">
+      <c r="AJ17" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="AK16" s="10" t="s">
+      <c r="AK17" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="AL16" s="10" t="s">
+      <c r="AL17" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="AM16" s="10" t="s">
+      <c r="AM17" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="AN16" s="10" t="s">
+      <c r="AN17" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="AO16" s="10" t="s">
+      <c r="AO17" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="AP16" s="10" t="s">
+      <c r="AP17" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="AQ16" s="10" t="s">
+      <c r="AQ17" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="AR16" s="10" t="s">
+      <c r="AR17" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="AS16" s="10" t="s">
+      <c r="AS17" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="AT16" s="10" t="s">
+      <c r="AT17" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="AU16" s="10" t="s">
+      <c r="AU17" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="AV16" s="10" t="s">
+      <c r="AV17" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AW16" s="10" t="s">
+      <c r="AW17" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="AX16" s="10"/>
-      <c r="AY16" s="10"/>
-      <c r="AZ16" s="10"/>
-    </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A17" s="17"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
-      <c r="N17" s="15"/>
-      <c r="O17" s="15"/>
-      <c r="P17" s="15"/>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="15"/>
-      <c r="S17" s="15"/>
-      <c r="T17" s="15"/>
-      <c r="U17" s="15"/>
-      <c r="V17" s="15"/>
-      <c r="W17" s="15"/>
-      <c r="X17" s="15"/>
-      <c r="Y17" s="15"/>
-      <c r="Z17" s="15"/>
-      <c r="AA17" s="15"/>
-      <c r="AB17" s="15"/>
-      <c r="AC17" s="15"/>
-      <c r="AD17" s="15"/>
-      <c r="AE17" s="16"/>
-      <c r="AF17" s="16"/>
-      <c r="AG17" s="16"/>
-      <c r="AH17" s="16"/>
-      <c r="AI17" s="15"/>
-      <c r="AJ17" s="15"/>
-      <c r="AK17" s="15"/>
-      <c r="AL17" s="15"/>
-      <c r="AM17" s="15"/>
-      <c r="AN17" s="15"/>
-      <c r="AO17" s="15"/>
-      <c r="AP17" s="15"/>
-      <c r="AQ17" s="15"/>
-      <c r="AR17" s="15"/>
-      <c r="AS17" s="15"/>
-      <c r="AT17" s="15"/>
-      <c r="AU17" s="15"/>
-      <c r="AV17" s="15"/>
-      <c r="AW17" s="28"/>
-      <c r="AX17" s="15"/>
-      <c r="AY17" s="15"/>
-      <c r="AZ17" s="15"/>
+      <c r="AX17" s="10"/>
+      <c r="AY17" s="10"/>
+      <c r="AZ17" s="10"/>
     </row>
     <row r="18" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
@@ -16302,7 +16267,7 @@
       <c r="AZ23" s="15"/>
     </row>
     <row r="24" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A24" s="18"/>
+      <c r="A24" s="17"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
@@ -16464,7 +16429,7 @@
       <c r="AZ26" s="15"/>
     </row>
     <row r="27" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A27" s="17"/>
+      <c r="A27" s="18"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
       <c r="D27" s="15"/>
@@ -17867,60 +17832,118 @@
       <c r="AY52" s="15"/>
       <c r="AZ52" s="15"/>
     </row>
+    <row r="53" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="A53" s="17"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
+      <c r="I53" s="15"/>
+      <c r="J53" s="15"/>
+      <c r="K53" s="15"/>
+      <c r="L53" s="15"/>
+      <c r="M53" s="15"/>
+      <c r="N53" s="15"/>
+      <c r="O53" s="15"/>
+      <c r="P53" s="15"/>
+      <c r="Q53" s="15"/>
+      <c r="R53" s="15"/>
+      <c r="S53" s="15"/>
+      <c r="T53" s="15"/>
+      <c r="U53" s="15"/>
+      <c r="V53" s="15"/>
+      <c r="W53" s="15"/>
+      <c r="X53" s="15"/>
+      <c r="Y53" s="15"/>
+      <c r="Z53" s="15"/>
+      <c r="AA53" s="15"/>
+      <c r="AB53" s="15"/>
+      <c r="AC53" s="15"/>
+      <c r="AD53" s="15"/>
+      <c r="AE53" s="16"/>
+      <c r="AF53" s="16"/>
+      <c r="AG53" s="16"/>
+      <c r="AH53" s="16"/>
+      <c r="AI53" s="15"/>
+      <c r="AJ53" s="15"/>
+      <c r="AK53" s="15"/>
+      <c r="AL53" s="15"/>
+      <c r="AM53" s="15"/>
+      <c r="AN53" s="15"/>
+      <c r="AO53" s="15"/>
+      <c r="AP53" s="15"/>
+      <c r="AQ53" s="15"/>
+      <c r="AR53" s="15"/>
+      <c r="AS53" s="15"/>
+      <c r="AT53" s="15"/>
+      <c r="AU53" s="15"/>
+      <c r="AV53" s="15"/>
+      <c r="AW53" s="28"/>
+      <c r="AX53" s="15"/>
+      <c r="AY53" s="15"/>
+      <c r="AZ53" s="15"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="B15:E15"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B12:E12"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B11:E11"/>
     <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B12:E12"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B7:E7"/>
   </mergeCells>
-  <dataValidations count="17">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="A value must be unique within the dataset" sqref="H17:H52" xr:uid="{274C493E-CBE0-2742-BFD6-A161E5736B5A}">
+  <dataValidations count="18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="A value must be unique within the dataset" sqref="H18:H53" xr:uid="{274C493E-CBE0-2742-BFD6-A161E5736B5A}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C17:C52" xr:uid="{792BC06D-75E6-1A4B-8EE7-26D8A0C4CF46}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C18:C53" xr:uid="{792BC06D-75E6-1A4B-8EE7-26D8A0C4CF46}">
       <formula1>"string,number,integer,boolean,array,object,timestamp,date,time,map,vector"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" sqref="B17:B52 J17:L52 O17:W52 Y17:AM52 AR17:AS52 AU17:AZ52" xr:uid="{DDC4FF9F-5023-E04B-9FAD-8E0C431863DF}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Is this a required field (true) or can it be optional (false)" sqref="G17:G52" xr:uid="{653181B6-028C-9348-B6A1-78F7EF7B9A52}">
+    <dataValidation allowBlank="1" sqref="B18:B53 J18:L53 O18:W53 Y18:AM53 AR18:AS53 AU18:AZ53" xr:uid="{DDC4FF9F-5023-E04B-9FAD-8E0C431863DF}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Is this a required field (true) or can it be optional (false)" sqref="G18:G53" xr:uid="{653181B6-028C-9348-B6A1-78F7EF7B9A52}">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Schema Name" prompt="The name of the schema (e.g., table) must match the Sheet name &quot;Schema &lt;schema_name&gt;&quot;" sqref="B5:E5" xr:uid="{8B3F718D-6361-B845-86DC-2F310C7348A9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Name of the property._x000a_If you have structured objects (child properties), use the dot notation, e.g., address.street._x000a_If you have array structures, use the [] notation, e.g., credit_cards[].number." sqref="A16" xr:uid="{0D2C99EC-1C07-E24C-A3B9-1D3DE4A213B3}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition Type" prompt="Type of definition for authority. Valid values are: businessDefinition, transformationImplementation, videoTutorial, tutorial, and implementation._x000a_ Maps to first authoritativeDefinitions.type_x000a_" sqref="N17:N52" xr:uid="{B83703A8-BFB7-EA4A-8244-28C8F1668E20}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Name of the property._x000a_If you have structured objects (child properties), use the dot notation, e.g., address.street._x000a_If you have array structures, use the [] notation, e.g., credit_cards[].number." sqref="A17" xr:uid="{0D2C99EC-1C07-E24C-A3B9-1D3DE4A213B3}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition Type" prompt="Type of definition for authority. Valid values are: businessDefinition, transformationImplementation, videoTutorial, tutorial, and implementation._x000a_ Maps to first authoritativeDefinitions.type_x000a_" sqref="N18:N53" xr:uid="{B83703A8-BFB7-EA4A-8244-28C8F1668E20}">
       <formula1>"businessDefinition,canonicalUrl,glossary,implementation,ontology,taxonomy,transformationImplementation,tutorial,videoTutorial"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I17:I52" xr:uid="{159197B4-47E7-9F48-923A-42F63EFB1F97}">
+    <dataValidation type="list" allowBlank="1" sqref="I18:I53" xr:uid="{159197B4-47E7-9F48-923A-42F63EFB1F97}">
       <formula1>"confidential,restricted,public"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition URL" prompt="Links to sources that provide more details on the element; examples would be a link to privacy statement, terms and conditions, license agreements, data catalog, or another tool._x000a__x000a_Maps to first authoritativeDefinitions.url_x000a_" sqref="M17:M52" xr:uid="{282580C6-13B6-1B40-9A3A-85842409A299}"/>
-    <dataValidation type="list" allowBlank="1" sqref="X17:X52" xr:uid="{17C32F0F-20AB-664B-ABCA-B45524F93539}">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition URL" prompt="Links to sources that provide more details on the element; examples would be a link to privacy statement, terms and conditions, license agreements, data catalog, or another tool._x000a__x000a_Maps to first authoritativeDefinitions.url_x000a_" sqref="M18:M53" xr:uid="{282580C6-13B6-1B40-9A3A-85842409A299}"/>
+    <dataValidation type="list" allowBlank="1" sqref="X18:X53" xr:uid="{17C32F0F-20AB-664B-ABCA-B45524F93539}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AW16" xr:uid="{D669647A-617C-7549-9EA2-AC37BFEA6E41}"/>
-    <dataValidation type="list" allowBlank="1" sqref="K17:K103" xr:uid="{FC6EF137-EF73-574C-95CF-B57336C59E8E}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AW17" xr:uid="{D669647A-617C-7549-9EA2-AC37BFEA6E41}"/>
+    <dataValidation type="list" allowBlank="1" sqref="K18:K104" xr:uid="{FC6EF137-EF73-574C-95CF-B57336C59E8E}">
       <formula1>"column,measure,dimension"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L17:L103 AQ17:AQ100 AT17:AT100" xr:uid="{A061E7B4-4C11-5241-BD09-1677165B8299}">
+    <dataValidation type="list" allowBlank="1" sqref="L18:L104 AQ18:AQ101 AT18:AT101" xr:uid="{A061E7B4-4C11-5241-BD09-1677165B8299}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:E14" xr:uid="{D05E7DD6-9150-B941-B705-FF6CFA22D7F9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B15:E15" xr:uid="{D05E7DD6-9150-B941-B705-FF6CFA22D7F9}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="AO17:AO100" xr:uid="{95DD2EA0-6986-414F-8048-0D9B55450EB2}">
+    <dataValidation type="list" allowBlank="1" sqref="AO18:AO101" xr:uid="{95DD2EA0-6986-414F-8048-0D9B55450EB2}">
       <formula1>"bfloat16,binary,float16,float32,float64,int8,uint8"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="AP17:AP100" xr:uid="{EF98B3E8-396D-0F48-A972-E0956219870A}">
+    <dataValidation type="list" allowBlank="1" sqref="AP18:AP101" xr:uid="{EF98B3E8-396D-0F48-A972-E0956219870A}">
       <formula1>"cosine,dotProduct,euclidean,hamming,manhattan"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="AN17:AN100" xr:uid="{F44F2772-48BF-B94D-9469-EC67E27A68CF}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="AN18:AN101" xr:uid="{F44F2772-48BF-B94D-9469-EC67E27A68CF}">
       <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:E7" xr:uid="{235F05D9-F9B3-6C48-A55D-32FE3C7AACA5}">
+      <formula1>"object,blob"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>